<commit_message>
Datos transaccionales ene-2025 a sep-2026 desde la base de órdenes de compra
- Fuente: base mensual completa de OC de Mercado Público (OC2025/OC2026), OC de
  convenio marco; se agrega sep-2026. Diferencia con lo publicado: +0,45%.
- Detalle de líneas, sector, ciudad y organismo para todos los meses.
- Selector de meses, tablas, gráficos y Excel actualizados (incluye sep-2026).
- Vista global: top 10 de proveedores por N° de OC y por monto por separado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oc-mensuales/administracion-y-entrega-de-beneficios/abr-2026.xlsx
+++ b/docs/oc-mensuales/administracion-y-entrega-de-beneficios/abr-2026.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Dirección de Educación, Doctrina e Historia de Car</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Dirección de Educación, Doctrina e Historia de Car</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Dirección de Educación, Doctrina e Historia de Carabineros</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Dirección General de Carabineros de Chile</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Dirección de Educación, Doctrina e Historia de Carabineros</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Bienes y Servicios</t>
+          <t>Hospital de Melipilla</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Dirección General de Carabineros de Chile</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD DEL MAULE HOSPITAL DE</t>
+          <t>Hospital de Constitución</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE LA SERENA</t>
+          <t>ILUSTRE MUNICIPALIDAD DE LA SERENA</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE LA SERENA</t>
+          <t>ILUSTRE MUNICIPALIDAD DE LA SERENA</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS XV ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Servicio Nacional del Patrimonio Cultural</t>
+          <t>SERVICIO NACIONAL DEL PATRIMONIO CULTURAL</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Regimiento Logístico N° 1 "Tocopilla"</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>COMISION CHILENA DE ENERGIA NUCLEAR</t>
+          <t>Comisión Chilena de Energía Nuclear</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3293,7 +3293,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Dirección de Educación, Doctrina e Historia de Carabineros</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>HOSPITAL CLAUDIO VICUNA</t>
+          <t>SERVICIO DE SALUD VALPARAISO SAN ANTONIO</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS VII ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -4334,7 +4334,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Carabineros de Chile - Dirección de Bienestar</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS I ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Araucanía</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Dirección General de Carabineros de Chile</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS ZONA SEG PRIV CONTROL ARMAS Y EXPL</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS ZONA SEG PRIV CONTROL ARMAS Y EXPL</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -5188,7 +5188,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Dirección General de Carabineros de Chile</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -5249,7 +5249,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS ZONA SEG PRIV CONTROL ARMAS Y EXPL</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -5310,7 +5310,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS ZONA SEG PRIV CONTROL ARMAS Y EXPL</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS ZONA SEG PRIV CONTROL ARMAS Y EXPL</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -5432,7 +5432,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS ZONA SEG PRIV CONTROL ARMAS Y EXPL</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -5676,7 +5676,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS ZONA SEG PRIV CONTROL ARMAS Y EXPL</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Dirección General de Carabineros de Chile</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -6042,7 +6042,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>DIRECCION REGIONAL DE ANTOFAGASTA</t>
+          <t>SERVICIO NACIONAL DEL PATRIMONIO CULTURAL</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -6103,7 +6103,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Servicio de Salud del Reloncaví</t>
+          <t>SERVICIO SALUD DEL RELONCAVI</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -6225,7 +6225,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Dirección General de Carabineros de Chile</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS ZONA SANTIAGO ESTE</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6530,7 +6530,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS IV ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -6713,7 +6713,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Consultorio General Urbano San Felipe</t>
+          <t>CONSULTORIO GENERAL URBANO SAN FELIPE</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -6774,7 +6774,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -6896,7 +6896,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>DIRECCIÓN REGIONAL DE COQUIMBO SERPAT</t>
+          <t>SERVICIO NACIONAL DEL PATRIMONIO CULTURAL</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -7018,7 +7018,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Dirección Regional de Gendarmeria - Temuco</t>
+          <t>DIRECCION GENERAL DE GENDARMERIA DE CHIL</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -7079,7 +7079,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>DIRECCIÓN REGIONAL DE COQUIMBO SERPAT</t>
+          <t>SERVICIO NACIONAL DEL PATRIMONIO CULTURAL</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -7384,7 +7384,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE QUIRIHUE</t>
+          <t>Ilustre Municipalidad de Quirihue</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -7872,7 +7872,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Servicio de Salud del Reloncaví</t>
+          <t>SERVICIO SALUD DEL RELONCAVI</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS X ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -8055,7 +8055,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS X ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -8177,7 +8177,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS X ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -8299,7 +8299,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS XI ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -8360,7 +8360,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>JEFATURA ADMINISTRATIVA Y LOGISTICA CAMPO MILITAR PENALOLEN</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -8482,7 +8482,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>REGIMIENTO 12 "SANGRA"</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS IX ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -8665,7 +8665,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS IX ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS IX ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -9397,7 +9397,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS XIV ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>DIRECCION REGIONAL DE VALPARAISO DEL SNPC</t>
+          <t>SERVICIO NACIONAL DEL PATRIMONIO CULTURAL</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -9580,7 +9580,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS II ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -9641,7 +9641,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS II ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -9702,7 +9702,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -10007,7 +10007,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Jefatura Adm y log Campo Militar Valdivia</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -10068,7 +10068,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -10373,7 +10373,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Servicio de Salud del Reloncaví</t>
+          <t>SERVICIO SALUD DEL RELONCAVI</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -10434,7 +10434,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Ilustre Municipalidad de Curanilahue - Salud</t>
+          <t>I MUNICIPALIDAD DE CURANILAHUE</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Dirección Regional de Gendarmeria - Valparaiso</t>
+          <t>DIRECCION GENERAL DE GENDARMERIA DE CHIL</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -10800,7 +10800,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Servicio de Salud del Reloncaví</t>
+          <t>SERVICIO SALUD DEL RELONCAVI</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Hospital de Achao</t>
+          <t>SERVICIO DE SALUD CHILOE</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Servicio Nacional del Patrimonio Cultural</t>
+          <t>SERVICIO NACIONAL DEL PATRIMONIO CULTURAL</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -11044,7 +11044,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -11166,7 +11166,7 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Zona de Bienestar Valdivia</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
@@ -11288,7 +11288,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Dirección Regional de Gendarmeria - Coyhaique</t>
+          <t>DIRECCION GENERAL DE GENDARMERIA DE CHIL</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
@@ -11349,7 +11349,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Dirección Regional de Gendarmeria - Antofagasta</t>
+          <t>DIRECCION GENERAL DE GENDARMERIA DE CHIL</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -11410,7 +11410,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS XVI ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -11593,7 +11593,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>Jefatura Adm. y Log. Campo Militar La Reina</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
@@ -11715,7 +11715,7 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS IX ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
@@ -11776,7 +11776,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -11837,7 +11837,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>COMISION CHILENA DE ENERGIA NUCLEAR</t>
+          <t>Comisión Chilena de Energía Nuclear</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
@@ -11898,7 +11898,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>JEFATURA ADMINISTRATIVA Y LOGISTICA DE LA GUARNICION COYHAIQUE</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -12020,7 +12020,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS I ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
@@ -12081,7 +12081,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS I ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -12264,7 +12264,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>Dirección General de Carabineros de Chile</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -12630,7 +12630,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>Jefatura Adm. y Log. de la División Logística</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
@@ -12996,7 +12996,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>EJERCITO DE CHILE</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
@@ -13179,7 +13179,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -13488,7 +13488,7 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>Dirección de Educación, Doctrina e Historia de Carabineros</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
@@ -13732,7 +13732,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>Carabineros de Chile - Unidad Contable Disalcar</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -13919,7 +13919,7 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE QUIRIHUE</t>
+          <t>Ilustre Municipalidad de Quirihue</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -14102,7 +14102,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -14163,7 +14163,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -14529,7 +14529,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Jefatura Adm y log Campo Militar Valdivia</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -15200,7 +15200,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>Departamento Provincial de Educación Osorno</t>
+          <t>SUBSECRETARIA DEL MINISTERIO DE EDUCACION PUBLICA</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -15261,7 +15261,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>Departamento Provincial de Educación Osorno</t>
+          <t>SUBSECRETARIA DEL MINISTERIO DE EDUCACION PUBLICA</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -15383,7 +15383,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS ZONA CARAB ARAUCANÍA CONT ORD PUBL</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>Carabineros de Chile</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
@@ -15505,7 +15505,7 @@
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>Carabineros de Chile</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -15566,7 +15566,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>Escuela de Gendarmeria</t>
+          <t>DIRECCION GENERAL DE GENDARMERIA DE CHIL</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -15810,7 +15810,7 @@
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>Comité de Seguro Agricola</t>
+          <t>Comité de Seguros del Agro</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
@@ -16241,7 +16241,7 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>VIII Zona de Carabineros Bio Bío</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
@@ -16607,7 +16607,7 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>Zona de Bienestar Valparaíso</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
@@ -16973,7 +16973,7 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>Servicio de Salud Atacama</t>
+          <t>SERVICIO DE SALUD ATACAMA</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
@@ -17095,7 +17095,7 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>Academia Politécnica Naval</t>
+          <t>DIRECCION DE ABASTECIMIENTO DE LA ARMADA</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
@@ -17156,7 +17156,7 @@
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>Academia Politécnica Naval</t>
+          <t>DIRECCION DE ABASTECIMIENTO DE LA ARMADA</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
@@ -17278,7 +17278,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS II ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -17339,7 +17339,7 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>Consultorio General Urbano Victor Domingo Silva</t>
+          <t>CONSULTORIO GENERAL URBANO VICTOR DOMINGO SILVA</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
@@ -17400,7 +17400,7 @@
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>JEFATURA ADMINISTRATIVA Y LOGISTICA CAMPO MILITAR PENALOLEN</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
@@ -17644,7 +17644,7 @@
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>Carabineros de Chile</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
@@ -17771,7 +17771,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -17827,7 +17827,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>SECCIÓN COMPRAS XV ZONA</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
@@ -17888,7 +17888,7 @@
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>COMISION CHILENA DE ENERGIA NUCLEAR</t>
+          <t>Comisión Chilena de Energía Nuclear</t>
         </is>
       </c>
       <c r="H286" t="inlineStr">
@@ -18076,7 +18076,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -18198,7 +18198,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -18437,7 +18437,7 @@
       </c>
       <c r="G295" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
@@ -18498,7 +18498,7 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
@@ -18620,7 +18620,7 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>Ejercito de Chile</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">

</xml_diff>

<commit_message>
Datos transaccionales: actualiza con las bases Parquet del 25-10-2026 (OC hasta el 24-10)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oc-mensuales/administracion-y-entrega-de-beneficios/abr-2026.xlsx
+++ b/docs/oc-mensuales/administracion-y-entrega-de-beneficios/abr-2026.xlsx
@@ -6254,7 +6254,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -19839,7 +19839,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">

</xml_diff>